<commit_message>
v0.1 of BRD finalised
</commit_message>
<xml_diff>
--- a/projects/phase-1-pre-sales-discovery/01-Presales-Discovery-Master-31072026.xlsx
+++ b/projects/phase-1-pre-sales-discovery/01-Presales-Discovery-Master-31072026.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d752cb73b61fc091/Desktop/linuxlabs/projectredstone/docs/project-management/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d752cb73b61fc091/Desktop/linuxlabs/projectredstone/projects/phase-1-pre-sales-discovery/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="99" documentId="8_{8FEB012A-8A23-45F5-8A6E-9B325831B842}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5387857-B7CA-4363-81CA-6F2FA390DD51}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4CDF954E-1E9A-4AFD-A2BB-B902DF9D4F7E}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4CDF954E-1E9A-4AFD-A2BB-B902DF9D4F7E}"/>
   </bookViews>
   <sheets>
     <sheet name="Discovery" sheetId="1" r:id="rId1"/>
@@ -1146,7 +1146,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
@@ -1274,10 +1274,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
@@ -1301,6 +1301,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1660,7 +1664,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="105" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="150" x14ac:dyDescent="0.25">
       <c r="A2" s="15">
         <v>1</v>
       </c>

</xml_diff>